<commit_message>
Update dashboard with audit fixes and highlighting feature
Changes:
- Q4 insight language revised for clarity
- Fixed 3 coding errors (Q2 R4, Q1 R9, Q1 R7)
- Cleaned _x000D_ artifacts from all response data
- Added code-to-text keyword highlighting feature
  - Click any code tag to highlight matching keywords
  - 151 keyword patterns for all codes
- Regenerated with corrected Excel data

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Alfaisal_Survey_Analysis.xlsx
+++ b/Alfaisal_Survey_Analysis.xlsx
@@ -585,9 +585,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -643,9 +640,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -689,9 +683,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -747,9 +738,6 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -793,9 +781,6 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
@@ -804,7 +789,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>Alfaisal University Case Study, MGT 490, Week 2, January 2026</t>
@@ -812,7 +796,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>Human-audited qualitative analysis of student survey responses</t>
@@ -5155,8 +5138,8 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>1- It has a very good reputation_x000D_
-2- You get to choose the major you want unlike public universities where there is competetion_x000D_
+          <t>1- It has a very good reputation 
+2- You get to choose the major you want unlike public universities where there is competetion 
 3- The student to faculty ratio is good, so there is better engagement in the class</t>
         </is>
       </c>
@@ -5334,8 +5317,8 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>reputation , because a lot of companies knows how high standard education is alfaisal so they might be more interested in._x000D_
-location , because alfaisal universty location is 5 minutes from my house ._x000D_
+          <t>reputation , because a lot of companies knows how high standard education is alfaisal so they might be more interested in. 
+location , because alfaisal universty location is 5 minutes from my house . 
 major ,entreprunuership and family busseniss major only availble at alfaisal .</t>
         </is>
       </c>
@@ -5405,7 +5388,9 @@
         <v>1</v>
       </c>
       <c r="H9" s="4" t="n"/>
-      <c r="I9" s="4" t="n"/>
+      <c r="I9" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
@@ -5433,7 +5418,11 @@
       <c r="AF9" s="4" t="n"/>
       <c r="AG9" s="4" t="n"/>
       <c r="AH9" s="4" t="n"/>
-      <c r="AI9" s="4" t="n"/>
+      <c r="AI9" s="4" t="inlineStr">
+        <is>
+          <t>Added: English: Instruction (was missing)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -5448,8 +5437,8 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>For it's Academic Reputation: Alfaisal is known for strong academic standards, English-meduim instruction, and reputable faculty, which increases the value of the degree in both local and international job markets._x000D_
-  Additionally, for it's career oppurtunity and major: I'm a finance student and alfaisal is known for it's partnerships, international orientation, and recognition in global rankings made it attractive for long-term career opportunities especially for students aiming to work in competitive sectors.</t>
+          <t>For it's Academic Reputation: Alfaisal is known for strong academic standards, English-meduim instruction, and reputable faculty, which increases the value of the degree in both local and international job markets. 
+ Additionally, for it's career oppurtunity and major: I'm a finance student and alfaisal is known for it's partnerships, international orientation, and recognition in global rankings made it attractive for long-term career opportunities especially for students aiming to work in competitive sectors.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -5462,7 +5451,9 @@
         <v>1</v>
       </c>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
+      <c r="H10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I10" s="4" t="n">
         <v>1</v>
       </c>
@@ -5472,7 +5463,9 @@
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="4" t="n"/>
       <c r="M10" s="4" t="n"/>
-      <c r="N10" s="4" t="n"/>
+      <c r="N10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O10" s="4" t="n"/>
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
@@ -5487,10 +5480,10 @@
       <c r="V10" s="4" t="n"/>
       <c r="W10" s="4" t="n"/>
       <c r="X10" s="4" t="n"/>
-      <c r="Y10" s="4" t="n"/>
-      <c r="Z10" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="4" t="n"/>
       <c r="AA10" s="4" t="n"/>
       <c r="AB10" s="4" t="n"/>
       <c r="AC10" s="4" t="n"/>
@@ -5499,7 +5492,11 @@
       <c r="AF10" s="4" t="n"/>
       <c r="AG10" s="4" t="n"/>
       <c r="AH10" s="4" t="n"/>
-      <c r="AI10" s="4" t="n"/>
+      <c r="AI10" s="4" t="inlineStr">
+        <is>
+          <t>Recoded: Added Partnerships, International Feel, Employment Outcomes; Removed Diversity (not mentioned)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -5514,7 +5511,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>In my opinion alfaisal university provides a community with a certain standard and prestiege that you wont find in other universities, this is an important point for building connections that could be useful in the future._x000D_
+          <t>In my opinion alfaisal university provides a community with a certain standard and prestiege that you wont find in other universities, this is an important point for building connections that could be useful in the future. 
 The other point is that Alfaisal provides one of the best and well respected degrees, that other universities would find hard to compete with.</t>
         </is>
       </c>
@@ -5878,8 +5875,8 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>One of the most significant factors that influenced our desicion to attend  is how active it seemed when we researched about it._x000D_
-  There were events offers such as competitors,career fairs,clubs,and a social enviroment that encourged networking.Another factor that influenced us is that Alfaisal established its reputation among the 9 private universities in Saudi Arabia. Weather through word of mouth or personal experience ,the reputation of Alfaisal sustained it self through the many graduates that has a sucssesful career.</t>
+          <t>One of the most significant factors that influenced our desicion to attend is how active it seemed when we researched about it. 
+ There were events offers such as competitors,career fairs,clubs,and a social enviroment that encourged networking.Another factor that influenced us is that Alfaisal established its reputation among the 9 private universities in Saudi Arabia. Weather through word of mouth or personal experience ,the reputation of Alfaisal sustained it self through the many graduates that has a sucssesful career.</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -6274,9 +6271,9 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>I chose alfaisal university for three main reasons._x000D_
-  First, it offers good acadimic quality in a smaller learning environment, which means better interaction with professors and more support._x000D_
-    Second, the university teaches in english and has students from different nationalitise.This helps prepare me for future carere opportunitiese.</t>
+          <t>I chose alfaisal university for three main reasons. 
+ First, it offers good acadimic quality in a smaller learning environment, which means better interaction with professors and more support. 
+  Second, the university teaches in english and has students from different nationalitise.This helps prepare me for future carere opportunitiese.</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
@@ -6545,8 +6542,8 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>1- My decision was based on a far family member that graduated with high grades and got oppurtunities straight ahead_x000D_
-  2- My goals alligne with the university way of learning, the university focuses and continious learning</t>
+          <t>1- My decision was based on a far family member that graduated with high grades and got oppurtunities straight ahead 
+ 2- My goals alligne with the university way of learning, the university focuses and continious learning</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
@@ -7345,7 +7342,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>We chose Alfaisal University for a variety of reasons; _x000D_
+          <t>We chose Alfaisal University for a variety of reasons; 
 One of the main reasons being is that it is the only university in Saudi Arabia which providing the OPM major (Operations Project Management). This would give us a competitive advantage in the market upon graduating. Alfaisal university also provides many career growth oppurtunities within this major such as the ability to test for the CAPM &amp; PMP certigicate prior to graduation. Social Factors is another reason for choosing this university, many of my cousins and siblings graduated from Alfaisal so there was some social pressure to join. The third reason is the location, Alfaisal University is only 15 minutes away from my house with some traffic, and around 30 mintes during rush hour making it convient to travel and arrive to my classess on time.</t>
         </is>
       </c>
@@ -8042,9 +8039,9 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Academic reputation, they are small but strong in quality and they have strong name education specily in business._x000D_
-  location they offer job oppertunites and they have lively culture._x000D_
-  social factors they support survive that enhance student life.</t>
+          <t>Academic reputation, they are small but strong in quality and they have strong name education specily in business. 
+ location they offer job oppertunites and they have lively culture. 
+ social factors they support survive that enhance student life.</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
@@ -8154,8 +8151,8 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>The main reason i chose alfaisal university for its academic reputation, english-medium instruction, and small class sizes . Alfaisal is known for high academic standards , and strong programs which made it appealing for students aiming for competitive careers _x000D_
-  The smaller learning envirornments also arouse for closer interactions with profersors</t>
+          <t>The main reason i chose alfaisal university for its academic reputation, english-medium instruction, and small class sizes . Alfaisal is known for high academic standards , and strong programs which made it appealing for students aiming for competitive careers 
+ The smaller learning envirornments also arouse for closer interactions with profersors</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
@@ -8214,13 +8211,13 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>From my prospective alfaisal university one of the top schools in saudi arabis because of the following reasons _x000D_
-  small, focused open culture _x000D_
-  strong local reputation _x000D_
-   english-medium instruction and international acadimic standers _x000D_
-  ability to combine the global knowlwdge with local relevance _x000D_
-  close link to the rop performance companies _x000D_
-  have some dividions like opreations and project managment that ai not provided by other university</t>
+          <t>From my prospective alfaisal university one of the top schools in saudi arabis because of the following reasons 
+ small, focused open culture 
+ strong local reputation 
+  english-medium instruction and international acadimic standers 
+ ability to combine the global knowlwdge with local relevance 
+ close link to the rop performance companies 
+ have some dividions like opreations and project managment that ai not provided by other university</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
@@ -9065,9 +9062,9 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>1- Alfaisal university has the best graduating employement in the whole country, and because most students only enter the university to get an education to get a job and alfaisal proves itself to be the best._x000D_
-    2- Alfaisal has a reputation of having one of the best staff and faculty and i always heard about their doctors and proffessors especially doctor julian._x000D_
-    3- A very big reason of why i joined alfaisal was because of the community it had, i thought about the connections i could have gotten if i had joined because i wanted to improve my social bubble.</t>
+          <t>1- Alfaisal university has the best graduating employement in the whole country, and because most students only enter the university to get an education to get a job and alfaisal proves itself to be the best. 
+  2- Alfaisal has a reputation of having one of the best staff and faculty and i always heard about their doctors and proffessors especially doctor julian. 
+  3- A very big reason of why i joined alfaisal was because of the community it had, i thought about the connections i could have gotten if i had joined because i wanted to improve my social bubble.</t>
         </is>
       </c>
       <c r="D75" s="4" t="n">
@@ -9124,9 +9121,9 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>1-) Alfaisal university has the best graduating employment in the whjole country, and because most students only enter the university to get an education to get a job and alfaisal proves itself to be the best._x000D_
-  2-) alfaisal has a reputation of having one of the best staff and faculty and before joining i always heard about their doctors and proffessors._x000D_
-  3-) a very big reason of why i joined alfaisal was because of the community it had, i thought about the connections i could have gotten if i had joined because i wanted to improve my social bubble.</t>
+          <t>1-) Alfaisal university has the best graduating employment in the whjole country, and because most students only enter the university to get an education to get a job and alfaisal proves itself to be the best. 
+ 2-) alfaisal has a reputation of having one of the best staff and faculty and before joining i always heard about their doctors and proffessors. 
+ 3-) a very big reason of why i joined alfaisal was because of the community it had, i thought about the connections i could have gotten if i had joined because i wanted to improve my social bubble.</t>
         </is>
       </c>
       <c r="D76" s="4" t="n">
@@ -9535,10 +9532,9 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>I chose alfaisal universty mainly because of its strong academic reputation, especially in business, and engineering, which prepares students for the global job market. The smaller class sizes also create a better learning experience and closer interaction with professoers._x000D_
-   _x000D_
-  Another important factor was the culture and enviroment. Alfaissl has a diverse student body, which helps devolp communication and teamwork skills in an international setting._x000D_
-    Lastly, its location in riyadh provides good internship and career opportunities while allowing me to stay close to my family.</t>
+          <t>I chose alfaisal universty mainly because of its strong academic reputation, especially in business, and engineering, which prepares students for the global job market. The smaller class sizes also create a better learning experience and closer interaction with professoers. 
+ Another important factor was the culture and enviroment. Alfaissl has a diverse student body, which helps devolp communication and teamwork skills in an international setting. 
+  Lastly, its location in riyadh provides good internship and career opportunities while allowing me to stay close to my family.</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
@@ -9819,9 +9815,9 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>1- Alfaisal University has the best graduating student employement in the whole country, and because most students enter university to get an education to ultimatily get a job Alfaisal proves itself to be the best._x000D_
-  2- Alfaisal has a community of the best students and a very strong staff and faculty which can prove essential for building a strong career in the future._x000D_
-  3- My father advised me to go to Alfaisal instead of King Saud University because Alfaisal has a very strong reputation in the job sector.</t>
+          <t>1- Alfaisal University has the best graduating student employement in the whole country, and because most students enter university to get an education to ultimatily get a job Alfaisal proves itself to be the best. 
+ 2- Alfaisal has a community of the best students and a very strong staff and faculty which can prove essential for building a strong career in the future. 
+ 3- My father advised me to go to Alfaisal instead of King Saud University because Alfaisal has a very strong reputation in the job sector.</t>
         </is>
       </c>
       <c r="D88" s="4" t="n">
@@ -10210,10 +10206,10 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>The top factors that influenced me to choose alfaisal was the following_x000D_
-    Better reputation and education quality compared to other universities in Riyadh region. The most important factor was the diversity of students amd professors allowing for room for more ideas and learning experiences form different cultures and backgrounds. _x000D_
-  Another factor was the location as it was very close to my house and i didnt have to waste my time and energy driving in the riyadh traffic, and could use my extra time for my benefit._x000D_
-  The faculty was kore respectful and cooperative at alfaisal and they kindly offered their assistance throughout the application process. The application and online services were smooth and easy to navigate compared to other universities where they was no clear application portal and the faculty was difficult to communicate with.</t>
+          <t>The top factors that influenced me to choose alfaisal was the following 
+  Better reputation and education quality compared to other universities in Riyadh region. The most important factor was the diversity of students amd professors allowing for room for more ideas and learning experiences form different cultures and backgrounds. 
+ Another factor was the location as it was very close to my house and i didnt have to waste my time and energy driving in the riyadh traffic, and could use my extra time for my benefit. 
+ The faculty was kore respectful and cooperative at alfaisal and they kindly offered their assistance throughout the application process. The application and online services were smooth and easy to navigate compared to other universities where they was no clear application portal and the faculty was difficult to communicate with.</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
@@ -10933,8 +10929,8 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>1) Alfaisal University has a good reputation and strong connections. This increases the chance of getting a good job after graduation._x000D_
-  2) Unlike many other universities, you're not obligated to register in the UPP program if you get good grades in the required examinations.</t>
+          <t>1) Alfaisal University has a good reputation and strong connections. This increases the chance of getting a good job after graduation. 
+ 2) Unlike many other universities, you're not obligated to register in the UPP program if you get good grades in the required examinations.</t>
         </is>
       </c>
       <c r="D107" s="4" t="n">
@@ -11215,8 +11211,8 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>1- Alfaisal university has a very good reputation and strong connections.This increase the chances of getting a decent job after graduation._x000D_
-  Unlike many other universities, in alfaisal uou are not obliged to do UPP program if you get good grades in high school, and required exams.</t>
+          <t>1- Alfaisal university has a very good reputation and strong connections.This increase the chances of getting a decent job after graduation. 
+ Unlike many other universities, in alfaisal uou are not obliged to do UPP program if you get good grades in high school, and required exams.</t>
         </is>
       </c>
       <c r="D112" s="4" t="n">
@@ -12077,16 +12073,18 @@
       <c r="R4" s="4" t="n"/>
       <c r="S4" s="4" t="n"/>
       <c r="T4" s="4" t="n"/>
-      <c r="U4" s="4" t="n"/>
+      <c r="U4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V4" s="4" t="n"/>
       <c r="W4" s="4" t="n"/>
       <c r="X4" s="4" t="n"/>
       <c r="Y4" s="4" t="n"/>
-      <c r="Z4" s="4" t="n"/>
+      <c r="Z4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="AA4" s="4" t="n"/>
-      <c r="AB4" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="AB4" s="4" t="n"/>
       <c r="AC4" s="4" t="n"/>
       <c r="AD4" s="4" t="n"/>
       <c r="AE4" s="4" t="n"/>
@@ -12094,7 +12092,11 @@
       <c r="AG4" s="4" t="n"/>
       <c r="AH4" s="4" t="n"/>
       <c r="AI4" s="4" t="n"/>
-      <c r="AJ4" s="4" t="n"/>
+      <c r="AJ4" s="4" t="inlineStr">
+        <is>
+          <t>Recoded: Family insisted on strong uni, not major choice</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -12457,7 +12459,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Another university is King saud university, since its considered as the university with the deepest root in saudi, and many well known polititians, coorprate founders and executives that graduated from there. _x000D_
+          <t>Another university is King saud university, since its considered as the university with the deepest root in saudi, and many well known polititians, coorprate founders and executives that graduated from there. 
 what made alfaisal uni stand out is that alfaisal is known for its community where only people who set high standards for themselves and their children send them there.</t>
         </is>
       </c>
@@ -12998,10 +13000,10 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>I considered King Saud University and princess Nourah Univirsity. Both are well known universities and offer good programs._x000D_
-  King Saud university has a strong reputation, but it is very large. I felt the classes might be too crowded._x000D_
-  Princess Nourah university was also a good option, but i wanted a more international environment._x000D_
-  Alfaisal won because it has smaller classes, teaches in english,and offers better interaction with professors.</t>
+          <t>I considered King Saud University and princess Nourah Univirsity. Both are well known universities and offer good programs. 
+ King Saud university has a strong reputation, but it is very large. I felt the classes might be too crowded. 
+ Princess Nourah university was also a good option, but i wanted a more international environment. 
+ Alfaisal won because it has smaller classes, teaches in english,and offers better interaction with professors.</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
@@ -14603,13 +14605,11 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>The other universities that I considered were all in the UK:_x000D_
-_x000D_
-King's College London _x000D_
-UCL _x000D_
-City University _x000D_
-University of Sussex- brighton_x000D_
-_x000D_
+          <t>The other universities that I considered were all in the UK: 
+King's College London 
+UCL 
+City University 
+University of Sussex- brighton 
 The reason why Alfaisal won, is because it is closer to home and it was an easy between the other local universities because, educationally, it sounded the most pleasing and i felt a sense of belonging to it. I was also pushed by my elder family members (my late grandmother's brother, we are very close he plays a grandfather figure in my life), so he adviced me since i was a Saudi who spent most of her life outside the kingdom, he said now is the best time to be in it. I had to build connections, professional or just platonic, with the people of my country.</t>
         </is>
       </c>
@@ -14788,8 +14788,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>one of the other universities i considered was prince sultan university, what made me consider prince sultan was that many of my friends attended that university and spoke highly of it, and it is also one of the highest ranked. But ultimately i didn't resonate with its social environment._x000D_
-_x000D_
+          <t>one of the other universities i considered was prince sultan university, what made me consider prince sultan was that many of my friends attended that university and spoke highly of it, and it is also one of the highest ranked. But ultimately i didn't resonate with its social environment. 
 i also wanted to study abroad and go to university college london, but that wasnt an option since, i graduated amidst covid.</t>
         </is>
       </c>
@@ -15290,10 +15289,10 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Prince Sultan University _x000D_
-  Sharjah University_x000D_
-  American University of Cairo_x000D_
-    Alfaisal University is actually not the first university I attended, as I briefly did a stint in a college in the US. Alfaisal University won because 1) it was more familiar amongst our family, 2) I would not need to move a second time, and 3) high school colleagues favored Alfaisal and could help me navigate as a student.</t>
+          <t>Prince Sultan University 
+ Sharjah University 
+ American University of Cairo 
+  Alfaisal University is actually not the first university I attended, as I briefly did a stint in a college in the US. Alfaisal University won because 1) it was more familiar amongst our family, 2) I would not need to move a second time, and 3) high school colleagues favored Alfaisal and could help me navigate as a student.</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
@@ -16015,8 +16014,8 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Prince Sultan university , King saud university_x000D_
-    Alfaisal won because its location was better than PSU and it gave me the major of my choice which KSU didn't do , alot of good talk of preffering alfaisal over PSU and i trusted it , The campus of alfaisal was the most welcome looking of both.</t>
+          <t>Prince Sultan university , King saud university 
+  Alfaisal won because its location was better than PSU and it gave me the major of my choice which KSU didn't do , alot of good talk of preffering alfaisal over PSU and i trusted it , The campus of alfaisal was the most welcome looking of both.</t>
         </is>
       </c>
       <c r="D75" s="4" t="n">
@@ -16190,10 +16189,9 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>I was considering princess noura for it being the largest women only university and having proper student accomodation and a lot cheaper than alfaisal, however the applying their was not a smooth process and it lacked diversity which was one of my concerns._x000D_
-   _x000D_
-  I also considered prince sultan but the faculty wasnt as respectful and helpful there and their was issues with their online system. Even thiug they had larger buildings and sports facilities, i did not feel connected to the environment their. Also the location was quite far which doesnt help as the traffic situation in Riyadh continues to rise._x000D_
-      I also applied to various international universities from chicago, london, turkey, and australia, and got accepted into most of them. After weighing out the pros and cons my parents decided to make me stay in Riyadh due to security and convinience.</t>
+          <t>I was considering princess noura for it being the largest women only university and having proper student accomodation and a lot cheaper than alfaisal, however the applying their was not a smooth process and it lacked diversity which was one of my concerns. 
+ I also considered prince sultan but the faculty wasnt as respectful and helpful there and their was issues with their online system. Even thiug they had larger buildings and sports facilities, i did not feel connected to the environment their. Also the location was quite far which doesnt help as the traffic situation in Riyadh continues to rise. 
+   I also applied to various international universities from chicago, london, turkey, and australia, and got accepted into most of them. After weighing out the pros and cons my parents decided to make me stay in Riyadh due to security and convinience.</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
@@ -17123,9 +17121,9 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Prince sultan university, but i faced some problems choosing it as the community in alfaisal is much better, newer classes and buildings._x000D_
-  Also, alfaisal won because of availability of all majors for femal students since prince sultan doesnt offer same majors for both genders._x000D_
-  Most important issue faced was that in prince sultan you are obligated to do the upp program.</t>
+          <t>Prince sultan university, but i faced some problems choosing it as the community in alfaisal is much better, newer classes and buildings. 
+ Also, alfaisal won because of availability of all majors for femal students since prince sultan doesnt offer same majors for both genders. 
+ Most important issue faced was that in prince sultan you are obligated to do the upp program.</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
@@ -17303,8 +17301,8 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>I wasnt actully sure what alfaisal university was I've never heard of it, I was actully considering studying enginerring at PSU (price sultan univeritsy) and I applied to PSU and got accepted there._x000D_
-  Why did alfaisal win? I had to sit with myself and questioned why did i want enginering and why i wanna study it, i did a lot of researching in the business field and discovered my passion and my intrests there, along with my research about business i came across a lot of articals talking about the top business schools in Riyadh, i went and asked around verious of people, who attended and how heard about them and iaxtully discovered it was the perfect choice for me and applied and got accepted</t>
+          <t>I wasnt actully sure what alfaisal university was I've never heard of it, I was actully considering studying enginerring at PSU (price sultan univeritsy) and I applied to PSU and got accepted there. 
+ Why did alfaisal win? I had to sit with myself and questioned why did i want enginering and why i wanna study it, i did a lot of researching in the business field and discovered my passion and my intrests there, along with my research about business i came across a lot of articals talking about the top business schools in Riyadh, i went and asked around verious of people, who attended and how heard about them and iaxtully discovered it was the perfect choice for me and applied and got accepted</t>
         </is>
       </c>
       <c r="D97" s="4" t="n">
@@ -18214,8 +18212,8 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Alfaisal's main competitive advantage lies in it's combination of high academic quality, international standards, and a small focused learning environment. _x000D_
-  It differentiates itself by offering globally oriented education within Saudi Arabia, supported by strong faculty, english instruction, and recognized rankings.</t>
+          <t>Alfaisal's main competitive advantage lies in it's combination of high academic quality, international standards, and a small focused learning environment. 
+ It differentiates itself by offering globally oriented education within Saudi Arabia, supported by strong faculty, english instruction, and recognized rankings.</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -18403,8 +18401,8 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>The thing the university offered like career fairs,events,ullumni relations._x000D_
-  How strong the university is academically</t>
+          <t>The thing the university offered like career fairs,events,ullumni relations. 
+ How strong the university is academically</t>
         </is>
       </c>
       <c r="D14" s="4" t="n"/>
@@ -19714,9 +19712,9 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Alfaisal's main source of competitive advntage is being the only private university that employers take seriously since they are strict with their ciriculum and grading.  _x000D_
-Its different from public universities becasue it doesn't require extremlly high grades in school and qudurat and those tests and because it teaches in english and that it accepts nonsaudi students. Its different from public universities because it has a strict program, a beautiful campus, and higher staff that respects students. _x000D_
-I considred PSU and alyamamah._x000D_
+          <t>Alfaisal's main source of competitive advntage is being the only private university that employers take seriously since they are strict with their ciriculum and grading.  
+Its different from public universities becasue it doesn't require extremlly high grades in school and qudurat and those tests and because it teaches in english and that it accepts nonsaudi students. Its different from public universities because it has a strict program, a beautiful campus, and higher staff that respects students. 
+I considred PSU and alyamamah. 
 Alfaisal won because it has it all, strict ciriculum, beautiful campus, and intelligent students.</t>
         </is>
       </c>
@@ -19983,11 +19981,10 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>We observed that Alfaisal's competitive advantage is it's ability to offer opportunities to its students consistently throughout its semesters. Students are exposed to some of the most prestigous companies in Saudi Arabia as early as their first year studying. Furthermore, as the faculty are highly experienced, they also can provide students with unique perspectives going into the workplace. _x000D_
-Creating value:_x000D_
-_x000D_
-Events_x000D_
-Alumni Relations_x000D_
+          <t>We observed that Alfaisal's competitive advantage is it's ability to offer opportunities to its students consistently throughout its semesters. Students are exposed to some of the most prestigous companies in Saudi Arabia as early as their first year studying. Furthermore, as the faculty are highly experienced, they also can provide students with unique perspectives going into the workplace. 
+Creating value: 
+Events 
+Alumni Relations 
 Clubs</t>
         </is>
       </c>
@@ -21122,8 +21119,8 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>They have good job hiering acceptance rate from the first year so they have a good reputation for both private and public sector companies so they give alot of good choices for their gradguates. They are different because they have the best facilities from my concideration and because they have the best study plan for business college._x000D_
-  I considered Prince sultan university and alyamamah university, but when I got my acceptance in Alfaisal university I was happy because it was my priority since most people I knew where in it from friends and family, and I heard good things from them.</t>
+          <t>They have good job hiering acceptance rate from the first year so they have a good reputation for both private and public sector companies so they give alot of good choices for their gradguates. They are different because they have the best facilities from my concideration and because they have the best study plan for business college. 
+ I considered Prince sultan university and alyamamah university, but when I got my acceptance in Alfaisal university I was happy because it was my priority since most people I knew where in it from friends and family, and I heard good things from them.</t>
         </is>
       </c>
       <c r="D67" s="4" t="n"/>
@@ -21651,8 +21648,8 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Alfaisal's main competitve advantage is it's student led environment. To add on, alfaisal being a smaller university gives it a stronger community where each student is able to recieve full attention from professors. _x000D_
-  On the contrary, prince sultan's enviorment is very strict, so more like a school rather than a university. In addition, PSU has a larger amount of students.</t>
+          <t>Alfaisal's main competitve advantage is it's student led environment. To add on, alfaisal being a smaller university gives it a stronger community where each student is able to recieve full attention from professors. 
+ On the contrary, prince sultan's enviorment is very strict, so more like a school rather than a university. In addition, PSU has a larger amount of students.</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
@@ -21822,10 +21819,10 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>- Close-knit campus culuter and supportive learning enviroment _x000D_
-  - Diverese international student community_x000D_
-  - Strong opportunities for networking and personal development _x000D_
-  - Modren facilities that improve student life, including the food court</t>
+          <t>- Close-knit campus culuter and supportive learning enviroment 
+ - Diverese international student community 
+ - Strong opportunities for networking and personal development 
+ - Modren facilities that improve student life, including the food court</t>
         </is>
       </c>
       <c r="D81" s="4" t="n"/>
@@ -22415,8 +22412,8 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Alfaisal university is considered mix with respect to our culture.It also holds beneficial mixed events which allows us to interact with the other gender in a way to prepare us for the job life. They hold different websites, such as simulations which helps us understand how the job life will look like._x000D_
-  They also take their students to events, and trips so we understand the material we are taking in classes and how it is implemented in real life, gets us good job oppurtinities and helps students make good connections.</t>
+          <t>Alfaisal university is considered mix with respect to our culture.It also holds beneficial mixed events which allows us to interact with the other gender in a way to prepare us for the job life. They hold different websites, such as simulations which helps us understand how the job life will look like. 
+ They also take their students to events, and trips so we understand the material we are taking in classes and how it is implemented in real life, gets us good job oppurtinities and helps students make good connections.</t>
         </is>
       </c>
       <c r="D92" s="4" t="n"/>
@@ -24300,8 +24297,8 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Yes, they are moderately threatened._x000D_
-    That is because some people's dream universities are going to be available in the near future, that can either be Arizona State of IE university, and they do not really have the facilities to apply for these universities that are outside the country, so they can be able to resort to these universities that are coming to the country.</t>
+          <t>Yes, they are moderately threatened. 
+  That is because some people's dream universities are going to be available in the near future, that can either be Arizona State of IE university, and they do not really have the facilities to apply for these universities that are outside the country, so they can be able to resort to these universities that are coming to the country.</t>
         </is>
       </c>
       <c r="D35" s="4" t="n"/>
@@ -24657,16 +24654,16 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>I belive yes to some extend but it will depend on the collages. _x000D_
-  I belive that the medcin collage will not be affected at all because they compete on the performance and they ranked as the best medicin school saudi arabia beeting all other university  and their students have 100 % sucess rate in the formal licen exam._x000D_
-  From the busniess school definitly they will got affected if they do not start to change. _x000D_
-  •  Some changes busniess school they can implement to sustain their comptitive advange:_x000D_
-  1- they need to change some of their faculty members_x000D_
-  2- they need to try to embeded some cources related to the technology espicallt that we are moving to service economy _x000D_
-  3- they need to redising how they teach channels. For example with the emergance of AI they need to use some apps like (sharpen provided by connect, which include vedios, flashcard, quizez) for some of the easy cuorses and moniter the performance and only let the student to come and have the formal exams. By doing that they can can cut the cost and reinvest that money in more excellent doctors _x000D_
-  4- they also have in involve more lab orianted teaching styles like simulation _x000D_
-  5- teach the student how to use AI tools as a hellping tool to help them how to make an informed, timly decasion when the information is not complete _x000D_
-  6- they should have substitute the grading for some subject like negotiation with pass or fail and make it harded more like real life pracice , to encourage the student to improve their skills even more, in you do not applay the knowledge to real life practive you will not pass</t>
+          <t>I belive yes to some extend but it will depend on the collages. 
+ I belive that the medcin collage will not be affected at all because they compete on the performance and they ranked as the best medicin school saudi arabia beeting all other university and their students have 100 % sucess rate in the formal licen exam. 
+ From the busniess school definitly they will got affected if they do not start to change. 
+ • Some changes busniess school they can implement to sustain their comptitive advange: 
+ 1- they need to change some of their faculty members 
+ 2- they need to try to embeded some cources related to the technology espicallt that we are moving to service economy 
+ 3- they need to redising how they teach channels. For example with the emergance of AI they need to use some apps like (sharpen provided by connect, which include vedios, flashcard, quizez) for some of the easy cuorses and moniter the performance and only let the student to come and have the formal exams. By doing that they can can cut the cost and reinvest that money in more excellent doctors 
+ 4- they also have in involve more lab orianted teaching styles like simulation 
+ 5- teach the student how to use AI tools as a hellping tool to help them how to make an informed, timly decasion when the information is not complete 
+ 6- they should have substitute the grading for some subject like negotiation with pass or fail and make it harded more like real life pracice , to encourage the student to improve their skills even more, in you do not applay the knowledge to real life practive you will not pass</t>
         </is>
       </c>
       <c r="D43" s="4" t="n"/>
@@ -26534,9 +26531,9 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>It depends on the prefences of the people._x000D_
-  In alfaisal university different languages  are being used in campus, which makes everyone feel like they are at home._x000D_
-  The teaching system is so strong and all doctors are very professional. Also, alfaisals community and campus is not so big which a lot of students and parents prefer as it is so safe and the security system is so strong.</t>
+          <t>It depends on the prefences of the people. 
+ In alfaisal university different languages are being used in campus, which makes everyone feel like they are at home. 
+ The teaching system is so strong and all doctors are very professional. Also, alfaisals community and campus is not so big which a lot of students and parents prefer as it is so safe and the security system is so strong.</t>
         </is>
       </c>
       <c r="D85" s="4" t="n"/>
@@ -27163,7 +27160,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>the main challenge i see is the faculty to students ratio, faculty includes all of the employees that work in campus including the technicians, janitors, etc..._x000D_
+          <t>the main challenge i see is the faculty to students ratio, faculty includes all of the employees that work in campus including the technicians, janitors, etc... 
 the main issue alfaisal strugles with is the amount of proffesors available for the students</t>
         </is>
       </c>
@@ -31067,7 +31064,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Knowlege &amp; Expirence Gained--&gt; While building a  sense of community--&gt; Gain Job Market Oppurtinities _x000D_
+          <t>Knowlege &amp; Expirence Gained--&gt; While building a sense of community--&gt; Gain Job Market Oppurtinities 
 Gaining knowlege &amp; expierence, while building a sense of community in order to gain job market opportunities</t>
         </is>
       </c>
@@ -31618,8 +31615,8 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Global standards, personalized education_x000D_
-Small, personal, globally competitive _x000D_
+          <t>Global standards, personalized education 
+Small, personal, globally competitive 
 quality over scale, globally alligned</t>
         </is>
       </c>
@@ -31662,9 +31659,9 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>- Global standards, personalized education_x000D_
-  - Small , personal, globally competitave_x000D_
-  - Quality over scale, globally alligned</t>
+          <t>- Global standards, personalized education 
+ - Small , personal, globally competitave 
+ - Quality over scale, globally alligned</t>
         </is>
       </c>
       <c r="D41" s="4" t="n">
@@ -31904,8 +31901,8 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>I think it all raedy has a great statement which is _x000D_
-  Shaping , Excellence, sustaining tomorrow</t>
+          <t>I think it all raedy has a great statement which is 
+ Shaping , Excellence, sustaining tomorrow</t>
         </is>
       </c>
       <c r="D47" s="4" t="n"/>
@@ -32599,8 +32596,8 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Give students a strong education, support and better career outcomes than competitors._x000D_
-  Keep Alfaisal high-quality and personal and focus on strong job opportunities for students.</t>
+          <t>Give students a strong education, support and better career outcomes than competitors. 
+ Keep Alfaisal high-quality and personal and focus on strong job opportunities for students.</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
@@ -32760,10 +32757,10 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>1: quality first, student always_x000D_
-  2: learn globally, succeed locally _x000D_
-  3: small classes, big futures _x000D_
-  4: eductate with purpose, complete with quality</t>
+          <t>1: quality first, student always 
+ 2: learn globally, succeed locally 
+ 3: small classes, big futures 
+ 4: eductate with purpose, complete with quality</t>
         </is>
       </c>
       <c r="D70" s="4" t="n">
@@ -32809,7 +32806,7 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>1- Keep Alfaisal high-quality and personal, and focus on strong job opportunities for students._x000D_
+          <t>1- Keep Alfaisal high-quality and personal, and focus on strong job opportunities for students. 
 2- Give students a strong education, personal support, and better career outcomes than competitors.</t>
         </is>
       </c>
@@ -32854,9 +32851,9 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>1. "Keep alfaisal high-quality and personal, and focus on strong job opportunities for students"._x000D_
-  2. "Stay a small, top-quality university in riyadh with great teaching and strong career support". _x000D_
-  3. "Give students a strong education, personal support, and better career outcomes thyan competitors".</t>
+          <t>1. "Keep alfaisal high-quality and personal, and focus on strong job opportunities for students". 
+ 2. "Stay a small, top-quality university in riyadh with great teaching and strong career support". 
+ 3. "Give students a strong education, personal support, and better career outcomes thyan competitors".</t>
         </is>
       </c>
       <c r="D72" s="4" t="n">
@@ -32904,9 +32901,9 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>1. "Keep Alfaisal high-quality and personal, and focus on strong job opportunities for students."_x000D_
-  2. "Stay a small, top-quality university in Riyadh with great teaching and strong career support."_x000D_
-  3. "Give students a strong education, personal support, and better career outcomes than competitors."</t>
+          <t>1. "Keep Alfaisal high-quality and personal, and focus on strong job opportunities for students." 
+ 2. "Stay a small, top-quality university in Riyadh with great teaching and strong career support." 
+ 3. "Give students a strong education, personal support, and better career outcomes than competitors."</t>
         </is>
       </c>
       <c r="D73" s="4" t="n">
@@ -32954,9 +32951,9 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>1- Keep Alfaisal high quality and personal, and focus on strong job opportunties for students_x000D_
-  2- Maintain the small size, top quality university in Riyadh with great teaching and strong career support_x000D_
-  3- Give students a strong education, personal and student support and better career outcome than competitors</t>
+          <t>1- Keep Alfaisal high quality and personal, and focus on strong job opportunties for students 
+ 2- Maintain the small size, top quality university in Riyadh with great teaching and strong career support 
+ 3- Give students a strong education, personal and student support and better career outcome than competitors</t>
         </is>
       </c>
       <c r="D74" s="4" t="n">
@@ -33160,8 +33157,8 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Knowledge, faith, and performance._x000D_
-  Prepare students to enter the job market and be the top among colleagues from other universities.</t>
+          <t>Knowledge, faith, and performance. 
+ Prepare students to enter the job market and be the top among colleagues from other universities.</t>
         </is>
       </c>
       <c r="D79" s="4" t="n"/>
@@ -33731,9 +33728,8 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1- partner with top companies to guarantee internships and real project for student _x000D_
-_x000D_
-2- upgrade faculty quality and bring more industry professionals to tech_x000D_
+          <t>1- partner with top companies to guarantee internships and real project for student 
+2- upgrade faculty quality and bring more industry professionals to tech 
 3- invest in labs , tech , and student support so the whole experience feels premiun</t>
         </is>
       </c>
@@ -33848,9 +33844,9 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1. Deepen industry partnerships to enhance internships _x000D_
-  2. Maintain small class size and strong faculty engagement _x000D_
-  3. Foucs on niche, high-demand programs aligned with vision 2030</t>
+          <t>1. Deepen industry partnerships to enhance internships 
+ 2. Maintain small class size and strong faculty engagement 
+ 3. Foucs on niche, high-demand programs aligned with vision 2030</t>
         </is>
       </c>
       <c r="D11" s="4" t="n"/>
@@ -34334,8 +34330,8 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>1.Evaluation of the education system, in order to rank higher and increase challanges in the curiculam therefore gaining a better reputation in the market_x000D_
-2. Possibly having more field trips and events to increase social interactions and building a sense of community _x000D_
+          <t>1.Evaluation of the education system, in order to rank higher and increase challanges in the curiculam therefore gaining a better reputation in the market 
+2. Possibly having more field trips and events to increase social interactions and building a sense of community 
 3. Both knowlege/skills gained throughout univeristy while building a sense of community and longlasting relationships/friendships (core memories) will enhance univesity expierence while stimultaneously preparing students to enter the job market with confidence and opportunities</t>
         </is>
       </c>
@@ -34598,8 +34594,8 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>1. Strengthen partnerships with industry to expand internships, projects, and career placment. _x000D_
-  2. Regular update curricula to meet international standards and market needs.</t>
+          <t>1. Strengthen partnerships with industry to expand internships, projects, and career placment. 
+ 2. Regular update curricula to meet international standards and market needs.</t>
         </is>
       </c>
       <c r="D31" s="4" t="n">
@@ -34643,9 +34639,9 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Improve interinship, indisrty partnership and develop strong colaprations with institution._x000D_
-  higher strong international doctors with modren teaching aproches._x000D_
-  focuse on student skills and employability.</t>
+          <t>Improve interinship, indisrty partnership and develop strong colaprations with institution. 
+ higher strong international doctors with modren teaching aproches. 
+ focuse on student skills and employability.</t>
         </is>
       </c>
       <c r="D32" s="4" t="n"/>
@@ -34681,7 +34677,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Instead of having "executive lecture" classes only in the last year of university, implement them throughout the years to futher familiarize students with the top companies in saudi early on._x000D_
+          <t>Instead of having "executive lecture" classes only in the last year of university, implement them throughout the years to futher familiarize students with the top companies in saudi early on. 
 Allowing students more workshops with the actual empolyees of said companies, properly preparing them in terms of CV, linkedins, soft skills, and technincal skills as well as allowing them field trips to the dominating companies in respective fields to expose them to the reality of work after studies.</t>
         </is>
       </c>
@@ -34790,9 +34786,9 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>1-Improve interniship,industry partnership and devlop strong collabrations with institution._x000D_
-  2- Higher strong international profassers with modren teaching approches._x000D_
-  3- Focus on students skills and employability.</t>
+          <t>1-Improve interniship,industry partnership and devlop strong collabrations with institution. 
+ 2- Higher strong international profassers with modren teaching approches. 
+ 3- Focus on students skills and employability.</t>
         </is>
       </c>
       <c r="D36" s="4" t="n"/>
@@ -34830,8 +34826,8 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Invest in flagship programs (medicine, business) _x000D_
-maintaining small class sizes _x000D_
+          <t>Invest in flagship programs (medicine, business) 
+maintaining small class sizes 
 build selective international partership</t>
         </is>
       </c>
@@ -34868,9 +34864,9 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>1- Invest in flagship programs ( medicine, business)_x000D_
-    2- Maintain small class sizes _x000D_
-    3- Build selective international partnership</t>
+          <t>1- Invest in flagship programs ( medicine, business) 
+  2- Maintain small class sizes 
+  3- Build selective international partnership</t>
         </is>
       </c>
       <c r="D38" s="4" t="n"/>
@@ -35236,9 +35232,9 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Teach more courses that explore international methodology (e..g International Finance, International Law, and International Culture)_x000D_
-    Provide more opportunties for students from around the world (by opening international scholarships, advertising to high schools around the world, and advertising to children of diplomats in Saudi Arabia.) _x000D_
-    Everybody in their respective colleges pay the same amount to attend the university.</t>
+          <t>Teach more courses that explore international methodology (e..g International Finance, International Law, and International Culture) 
+  Provide more opportunties for students from around the world (by opening international scholarships, advertising to high schools around the world, and advertising to children of diplomats in Saudi Arabia.) 
+  Everybody in their respective colleges pay the same amount to attend the university.</t>
         </is>
       </c>
       <c r="D48" s="4" t="n"/>
@@ -35570,8 +35566,8 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>1_x000D_
-  Market scholarships for students getting specific grades , get skilled instructirs by first satsfying your existing ones with pay and everything , buy nearby land and expand or do more floors and market and advertise everything.</t>
+          <t>1 
+ Market scholarships for students getting specific grades , get skilled instructirs by first satsfying your existing ones with pay and everything , buy nearby land and expand or do more floors and market and advertise everything.</t>
         </is>
       </c>
       <c r="D57" s="4" t="n"/>
@@ -36151,8 +36147,8 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Experience faculty, good learning system, having labs that meets the needs of the majors._x000D_
-  When students start the coop training , they keep incontact with the students and every student gets assigned to an advisor that monitor and guides the student through their journey</t>
+          <t>Experience faculty, good learning system, having labs that meets the needs of the majors. 
+ When students start the coop training , they keep incontact with the students and every student gets assigned to an advisor that monitor and guides the student through their journey</t>
         </is>
       </c>
       <c r="D72" s="4" t="n"/>

</xml_diff>